<commit_message>
APS PURAN v2.0 - interface profissional, cadastros inline e correções
</commit_message>
<xml_diff>
--- a/ENTREGAS/APS_PURAN_FINAL.xlsx
+++ b/ENTREGAS/APS_PURAN_FINAL.xlsx
@@ -29,7 +29,7 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy hh:mm"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -72,8 +72,37 @@
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font/>
   </fonts>
-  <fills count="11">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -134,8 +163,50 @@
         <bgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+        <bgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+        <bgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C55A11"/>
+        <bgColor rgb="00C55A11"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+        <bgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E7E6E6"/>
+        <bgColor rgb="00E7E6E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C00000"/>
+        <bgColor rgb="00C00000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -171,11 +242,99 @@
         <color rgb="002E75B6"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="002E75B6"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="002E75B6"/>
+      </right>
+      <top style="medium">
+        <color rgb="002E75B6"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="002E75B6"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="002E75B6"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="002E75B6"/>
+      </right>
+      <top style="medium">
+        <color rgb="002E75B6"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="002E75B6"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -251,6 +410,94 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -618,114 +865,157 @@
   </sheetPr>
   <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="35" customHeight="1">
+      <c r="A1" s="27" t="inlineStr">
         <is>
           <t>APS PURAN</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="28" t="inlineStr">
         <is>
           <t>Sistema de Planejamento e Controle da Produção  |  23/08/2026 05:43</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="29" t="inlineStr">
         <is>
           <t>STATUS: OPERACIONAL</t>
         </is>
       </c>
     </row>
+    <row r="4" ht="25" customHeight="1">
+      <c r="A4" s="30" t="n"/>
+      <c r="C4" s="30" t="n"/>
+      <c r="E4" s="30" t="n"/>
+      <c r="G4" s="30" t="n"/>
+    </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="31" t="inlineStr">
         <is>
           <t>TOTAL DE OPs</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="B5" s="32" t="n"/>
+      <c r="C5" s="31" t="inlineStr">
         <is>
           <t>EM PRODUÇÃO</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="D5" s="32" t="n"/>
+      <c r="E5" s="31" t="inlineStr">
         <is>
           <t>ATRASADAS</t>
         </is>
       </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="F5" s="32" t="n"/>
+      <c r="G5" s="31" t="inlineStr">
         <is>
           <t>CONCLUÍDAS</t>
         </is>
       </c>
-    </row>
-    <row r="6">
+      <c r="H5" s="32" t="n"/>
+    </row>
+    <row r="6" ht="25" customHeight="1">
       <c r="A6" s="8">
         <f>COUNTA(DADOS!A:A)-1</f>
         <v/>
       </c>
+      <c r="B6" s="32" t="n"/>
       <c r="C6" s="8">
         <f>COUNTIF(DADOS!S:S,"EM PRODUÇÃO")</f>
         <v/>
       </c>
+      <c r="D6" s="32" t="n"/>
       <c r="E6" s="8">
         <f>COUNTIF(DADOS!S:S,"ATRASADO")</f>
         <v/>
       </c>
+      <c r="F6" s="32" t="n"/>
       <c r="G6" s="8">
         <f>COUNTIF(DADOS!S:S,"CONCLUÍDO")</f>
         <v/>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="H6" s="32" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="33" t="n"/>
+      <c r="C7" s="33" t="n"/>
+      <c r="E7" s="33" t="n"/>
+      <c r="G7" s="33" t="n"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="34" t="inlineStr">
         <is>
           <t>TOTAL CAIXAS</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>HORAS PLANEJADAS</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>HORAS ATRASO</t>
-        </is>
-      </c>
-      <c r="G8" s="10" t="inlineStr">
-        <is>
-          <t>OPs C/ ATRASO</t>
-        </is>
-      </c>
+      <c r="B8" s="35" t="n"/>
+      <c r="C8" s="35" t="n"/>
+      <c r="D8" s="35" t="n"/>
+      <c r="E8" s="35" t="n"/>
+      <c r="F8" s="35" t="n"/>
+      <c r="G8" s="35" t="n"/>
+      <c r="H8" s="32" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="8">
+      <c r="A9" s="36">
         <f>SUM(DADOS!F:F)</f>
         <v/>
       </c>
-      <c r="C9" s="8">
+      <c r="B9" s="37" t="n"/>
+      <c r="C9" s="36">
         <f>SUM(DADOS!P:P)</f>
         <v/>
       </c>
-      <c r="E9" s="8">
+      <c r="D9" s="37" t="n"/>
+      <c r="E9" s="36">
         <f>SUM(DADOS!T:T)</f>
         <v/>
       </c>
-      <c r="G9" s="8">
+      <c r="F9" s="37" t="n"/>
+      <c r="G9" s="36">
         <f>COUNTIF(DADOS!T:T,"&gt;0")</f>
         <v/>
       </c>
+      <c r="H9" s="37" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="38" t="n"/>
+      <c r="B10" s="38" t="n"/>
+      <c r="C10" s="38" t="n"/>
+      <c r="D10" s="38" t="n"/>
+      <c r="E10" s="38" t="n"/>
+      <c r="F10" s="38" t="n"/>
+      <c r="G10" s="38" t="n"/>
+      <c r="H10" s="38" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="39" t="inlineStr">
         <is>
           <t>ALERTAS E NOTIFICAÇÕES</t>
         </is>
       </c>
+      <c r="B11" s="38" t="n"/>
+      <c r="C11" s="38" t="n"/>
+      <c r="D11" s="38" t="n"/>
+      <c r="E11" s="38" t="n"/>
+      <c r="F11" s="38" t="n"/>
+      <c r="G11" s="38" t="n"/>
+      <c r="H11" s="38" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
@@ -733,9 +1023,23 @@
           <t>• Nenhuma alerta no momento</t>
         </is>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="12" t="inlineStr"/>
+      <c r="B12" s="35" t="n"/>
+      <c r="C12" s="35" t="n"/>
+      <c r="D12" s="35" t="n"/>
+      <c r="E12" s="35" t="n"/>
+      <c r="F12" s="35" t="n"/>
+      <c r="G12" s="35" t="n"/>
+      <c r="H12" s="32" t="n"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="40" t="inlineStr"/>
+      <c r="B13" s="35" t="n"/>
+      <c r="C13" s="35" t="n"/>
+      <c r="D13" s="35" t="n"/>
+      <c r="E13" s="35" t="n"/>
+      <c r="F13" s="35" t="n"/>
+      <c r="G13" s="35" t="n"/>
+      <c r="H13" s="32" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
@@ -743,6 +1047,13 @@
           <t>• O sistema está operacional</t>
         </is>
       </c>
+      <c r="B14" s="35" t="n"/>
+      <c r="C14" s="35" t="n"/>
+      <c r="D14" s="35" t="n"/>
+      <c r="E14" s="35" t="n"/>
+      <c r="F14" s="35" t="n"/>
+      <c r="G14" s="35" t="n"/>
+      <c r="H14" s="32" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
@@ -750,6 +1061,13 @@
           <t>• Clique nos botões abaixo para acessar as funcionalidades</t>
         </is>
       </c>
+      <c r="B15" s="35" t="n"/>
+      <c r="C15" s="35" t="n"/>
+      <c r="D15" s="35" t="n"/>
+      <c r="E15" s="35" t="n"/>
+      <c r="F15" s="35" t="n"/>
+      <c r="G15" s="35" t="n"/>
+      <c r="H15" s="32" t="n"/>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="11" t="inlineStr">
@@ -764,11 +1082,17 @@
           <t>📅 PLANEJAMENTO</t>
         </is>
       </c>
+      <c r="B20" s="41" t="n"/>
+      <c r="C20" s="41" t="n"/>
+      <c r="D20" s="42" t="n"/>
       <c r="E20" s="13" t="inlineStr">
         <is>
           <t>📋 OPERAÇÕES</t>
         </is>
       </c>
+      <c r="F20" s="41" t="n"/>
+      <c r="G20" s="41" t="n"/>
+      <c r="H20" s="42" t="n"/>
     </row>
     <row r="22" ht="6.666666666666667" customHeight="1">
       <c r="A22" s="13" t="inlineStr">
@@ -776,14 +1100,20 @@
           <t>⚙ MÁQUINAS</t>
         </is>
       </c>
+      <c r="B22" s="41" t="n"/>
+      <c r="C22" s="41" t="n"/>
+      <c r="D22" s="42" t="n"/>
       <c r="E22" s="13" t="inlineStr">
         <is>
           <t>🔎 PESQUISAR OP</t>
         </is>
       </c>
+      <c r="F22" s="41" t="n"/>
+      <c r="G22" s="41" t="n"/>
+      <c r="H22" s="42" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="29">
+  <mergeCells count="30">
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A15:H15"/>
     <mergeCell ref="A22:D22"/>
@@ -809,6 +1139,7 @@
     <mergeCell ref="E20:H20"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A8:H8"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="A13:H13"/>
     <mergeCell ref="A9:B9"/>
@@ -838,29 +1169,29 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Z11"/>
+  <dimension ref="A1:Z14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
-    <col width="16" customWidth="1" min="17" max="17"/>
-    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
     <col width="14" customWidth="1" min="19" max="19"/>
-    <col width="10" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
     <col width="10" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="16" customWidth="1" min="23" max="23"/>
@@ -868,22 +1199,22 @@
     <col width="25" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
-    <row r="1" ht="35" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="43" t="inlineStr">
         <is>
           <t>OPERAÇÕES</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="14" t="inlineStr">
+      <c r="A2" s="28" t="inlineStr">
         <is>
           <t>Gestão de ordens de produção</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="44" t="inlineStr">
         <is>
           <t>🔎 PESQUISAR OP</t>
         </is>
@@ -915,37 +1246,55 @@
       </c>
       <c r="H5" s="17" t="n"/>
     </row>
-    <row r="7">
-      <c r="A7" s="15" t="inlineStr">
-        <is>
-          <t>AÇÕES</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>+ NOVA OP</t>
-        </is>
-      </c>
+    <row r="6">
+      <c r="A6" s="45" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="46" t="inlineStr">
+        <is>
+          <t>Numero da OP:</t>
+        </is>
+      </c>
+      <c r="B7" s="47" t="n"/>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="48" t="inlineStr">
+        <is>
+          <t>Produto:</t>
+        </is>
+      </c>
+      <c r="B8" s="49" t="n"/>
+      <c r="C8" s="42" t="n"/>
       <c r="D8" s="18" t="inlineStr">
         <is>
           <t>🔄 ATUALIZAR</t>
         </is>
       </c>
+      <c r="E8" s="41" t="n"/>
+      <c r="F8" s="42" t="n"/>
       <c r="G8" s="18" t="inlineStr">
         <is>
           <t>← VOLTAR</t>
         </is>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>OP</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="H8" s="41" t="n"/>
+      <c r="I8" s="42" t="n"/>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="50" t="inlineStr">
+        <is>
+          <t>Maquina:</t>
+        </is>
+      </c>
+      <c r="B9" s="47" t="n"/>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="51" t="inlineStr">
+        <is>
+          <t>Quantidade:</t>
+        </is>
+      </c>
+      <c r="B10" s="52" t="inlineStr">
         <is>
           <t>Produto</t>
         </is>
@@ -1066,13 +1415,13 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>OP001</t>
-        </is>
-      </c>
-      <c r="B11" s="19" t="inlineStr">
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="53" t="inlineStr">
+        <is>
+          <t>Unidade:</t>
+        </is>
+      </c>
+      <c r="B11" s="54" t="inlineStr">
         <is>
           <t>PURAN</t>
         </is>
@@ -1149,15 +1498,34 @@
       <c r="X11" s="19" t="inlineStr"/>
       <c r="Y11" s="12" t="inlineStr"/>
     </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="55" t="inlineStr">
+        <is>
+          <t>SALVAR OP</t>
+        </is>
+      </c>
+      <c r="C12" s="56" t="inlineStr">
+        <is>
+          <t>CANCELAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="57" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="11">
+    <mergeCell ref="C12:D12"/>
     <mergeCell ref="A1:Z1"/>
     <mergeCell ref="A7:H7"/>
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="G8:I8"/>
+    <mergeCell ref="A6:E6"/>
     <mergeCell ref="A2:Z2"/>
     <mergeCell ref="D8:F8"/>
+    <mergeCell ref="A14:T14"/>
+    <mergeCell ref="A12:B12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -1170,47 +1538,60 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Z9"/>
+  <dimension ref="A1:Z13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="35" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="43" t="inlineStr">
         <is>
           <t>MÁQUINAS</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="14" t="inlineStr">
+      <c r="A2" s="28" t="inlineStr">
         <is>
           <t>Gestão de recursos produtivos</t>
         </is>
       </c>
     </row>
     <row r="4" ht="25" customHeight="1">
-      <c r="A4" s="23" t="inlineStr">
+      <c r="A4" s="58" t="inlineStr">
         <is>
           <t>+ NOVA MÁQUINA</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Máquina</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B4" s="41" t="n"/>
+      <c r="C4" s="41" t="n"/>
+      <c r="D4" s="41" t="n"/>
+      <c r="E4" s="41" t="n"/>
+      <c r="F4" s="42" t="n"/>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="50" t="inlineStr">
+        <is>
+          <t>Codigo:</t>
+        </is>
+      </c>
+      <c r="B5" s="47" t="n"/>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="51" t="inlineStr">
+        <is>
+          <t>Nome:</t>
+        </is>
+      </c>
+      <c r="B6" s="52" t="inlineStr">
         <is>
           <t>Velocidade</t>
         </is>
@@ -1246,13 +1627,13 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="19" t="inlineStr">
-        <is>
-          <t>FETTE 2090</t>
-        </is>
-      </c>
-      <c r="B7" s="21" t="n">
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="53" t="inlineStr">
+        <is>
+          <t>Velocidade (cx/h):</t>
+        </is>
+      </c>
+      <c r="B7" s="59" t="n">
         <v>500</v>
       </c>
       <c r="C7" s="21" t="inlineStr">
@@ -1280,13 +1661,13 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="19" t="inlineStr">
-        <is>
-          <t>FETTE 2</t>
-        </is>
-      </c>
-      <c r="B8" s="21" t="n">
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="53" t="inlineStr">
+        <is>
+          <t>OEE (%):</t>
+        </is>
+      </c>
+      <c r="B8" s="59" t="n">
         <v>450</v>
       </c>
       <c r="C8" s="21" t="inlineStr">
@@ -1314,13 +1695,13 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>MEDISEAL</t>
-        </is>
-      </c>
-      <c r="B9" s="21" t="n">
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="53" t="inlineStr">
+        <is>
+          <t>Setup (h):</t>
+        </is>
+      </c>
+      <c r="B9" s="59" t="n">
         <v>600</v>
       </c>
       <c r="C9" s="21" t="inlineStr">
@@ -1348,9 +1729,27 @@
         </is>
       </c>
     </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="55" t="inlineStr">
+        <is>
+          <t>SALVAR MAQUINA</t>
+        </is>
+      </c>
+      <c r="C11" s="56" t="inlineStr">
+        <is>
+          <t>CANCELAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="57" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="6">
     <mergeCell ref="A1:Z1"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A13:H13"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="A2:Z2"/>
   </mergeCells>
@@ -1365,7 +1764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AW9"/>
+  <dimension ref="A1:CU9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1419,19 +1818,70 @@
     <col width="9" customWidth="1" min="49" max="49"/>
   </cols>
   <sheetData>
-    <row r="1" ht="35" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="43" t="inlineStr">
         <is>
           <t>PLANEJAMENTO DA PRODUÇÃO</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="14" t="inlineStr">
+      <c r="A2" s="28" t="inlineStr">
         <is>
           <t>Timeline visual e cards das OPs</t>
         </is>
       </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="60" t="n"/>
+      <c r="B3" s="60" t="n"/>
+      <c r="C3" s="60" t="n"/>
+      <c r="D3" s="60" t="n"/>
+      <c r="E3" s="60" t="n"/>
+      <c r="F3" s="60" t="n"/>
+      <c r="G3" s="60" t="n"/>
+      <c r="H3" s="60" t="n"/>
+      <c r="I3" s="60" t="n"/>
+      <c r="J3" s="60" t="n"/>
+      <c r="K3" s="60" t="n"/>
+      <c r="L3" s="60" t="n"/>
+      <c r="M3" s="60" t="n"/>
+      <c r="N3" s="60" t="n"/>
+      <c r="O3" s="60" t="n"/>
+      <c r="P3" s="60" t="n"/>
+      <c r="Q3" s="60" t="n"/>
+      <c r="R3" s="60" t="n"/>
+      <c r="S3" s="60" t="n"/>
+      <c r="T3" s="60" t="n"/>
+      <c r="U3" s="60" t="n"/>
+      <c r="V3" s="60" t="n"/>
+      <c r="W3" s="60" t="n"/>
+      <c r="X3" s="60" t="n"/>
+      <c r="Y3" s="60" t="n"/>
+      <c r="Z3" s="60" t="n"/>
+      <c r="AA3" s="60" t="n"/>
+      <c r="AB3" s="60" t="n"/>
+      <c r="AC3" s="60" t="n"/>
+      <c r="AD3" s="60" t="n"/>
+      <c r="AE3" s="60" t="n"/>
+      <c r="AF3" s="60" t="n"/>
+      <c r="AG3" s="60" t="n"/>
+      <c r="AH3" s="60" t="n"/>
+      <c r="AI3" s="60" t="n"/>
+      <c r="AJ3" s="60" t="n"/>
+      <c r="AK3" s="60" t="n"/>
+      <c r="AL3" s="60" t="n"/>
+      <c r="AM3" s="60" t="n"/>
+      <c r="AN3" s="60" t="n"/>
+      <c r="AO3" s="60" t="n"/>
+      <c r="AP3" s="60" t="n"/>
+      <c r="AQ3" s="60" t="n"/>
+      <c r="AR3" s="60" t="n"/>
+      <c r="AS3" s="60" t="n"/>
+      <c r="AT3" s="60" t="n"/>
+      <c r="AU3" s="60" t="n"/>
+      <c r="AV3" s="60" t="n"/>
+      <c r="AW3" s="60" t="n"/>
     </row>
     <row r="4" ht="25" customHeight="1">
       <c r="A4" s="18" t="inlineStr">
@@ -1439,6 +1889,21 @@
           <t>🔄 RECALCULAR  ⚠ ATRASOS  🔧 EVENTOS  🍽 REFEIÇÕES  🏠 DASHBOARD</t>
         </is>
       </c>
+      <c r="B4" s="41" t="n"/>
+      <c r="C4" s="41" t="n"/>
+      <c r="D4" s="41" t="n"/>
+      <c r="E4" s="41" t="n"/>
+      <c r="F4" s="41" t="n"/>
+      <c r="G4" s="41" t="n"/>
+      <c r="H4" s="41" t="n"/>
+      <c r="I4" s="41" t="n"/>
+      <c r="J4" s="41" t="n"/>
+      <c r="K4" s="41" t="n"/>
+      <c r="L4" s="41" t="n"/>
+      <c r="M4" s="41" t="n"/>
+      <c r="N4" s="41" t="n"/>
+      <c r="O4" s="41" t="n"/>
+      <c r="P4" s="42" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="25" t="inlineStr">
@@ -1709,8 +2174,10 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="5">
+    <mergeCell ref="A2:CU2"/>
     <mergeCell ref="A1:Z1"/>
+    <mergeCell ref="A1:CU1"/>
     <mergeCell ref="A4:P4"/>
     <mergeCell ref="A2:Z2"/>
   </mergeCells>

</xml_diff>

<commit_message>
APS PURAN - sincronizar planilha final em ENTREGAS/
</commit_message>
<xml_diff>
--- a/ENTREGAS/APS_PURAN_FINAL.xlsx
+++ b/ENTREGAS/APS_PURAN_FINAL.xlsx
@@ -29,7 +29,7 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy hh:mm"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -72,37 +72,8 @@
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="18"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001F4E78"/>
-      <sz val="16"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="16"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font/>
   </fonts>
-  <fills count="18">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -163,50 +134,8 @@
         <bgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-        <bgColor rgb="001F4E78"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
-        <bgColor rgb="00D9E1F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C55A11"/>
-        <bgColor rgb="00C55A11"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
-        <bgColor rgb="00FCE4D6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="004472C4"/>
-        <bgColor rgb="004472C4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E7E6E6"/>
-        <bgColor rgb="00E7E6E6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C00000"/>
-        <bgColor rgb="00C00000"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="11">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -242,99 +171,11 @@
         <color rgb="002E75B6"/>
       </bottom>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00CCCCCC"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00CCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CCCCCC"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00CCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00CCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="002E75B6"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="002E75B6"/>
-      </right>
-      <top style="medium">
-        <color rgb="002E75B6"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="002E75B6"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="002E75B6"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="002E75B6"/>
-      </right>
-      <top style="medium">
-        <color rgb="002E75B6"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="002E75B6"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -410,94 +251,6 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -865,157 +618,114 @@
   </sheetPr>
   <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-  </cols>
   <sheetData>
-    <row r="1" ht="35" customHeight="1">
-      <c r="A1" s="27" t="inlineStr">
+    <row r="1" ht="40" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>APS PURAN</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="28" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Sistema de Planejamento e Controle da Produção  |  23/08/2026 05:43</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="29" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>STATUS: OPERACIONAL</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="25" customHeight="1">
-      <c r="A4" s="30" t="n"/>
-      <c r="C4" s="30" t="n"/>
-      <c r="E4" s="30" t="n"/>
-      <c r="G4" s="30" t="n"/>
-    </row>
     <row r="5">
-      <c r="A5" s="31" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>TOTAL DE OPs</t>
         </is>
       </c>
-      <c r="B5" s="32" t="n"/>
-      <c r="C5" s="31" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>EM PRODUÇÃO</t>
         </is>
       </c>
-      <c r="D5" s="32" t="n"/>
-      <c r="E5" s="31" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>ATRASADAS</t>
         </is>
       </c>
-      <c r="F5" s="32" t="n"/>
-      <c r="G5" s="31" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
         <is>
           <t>CONCLUÍDAS</t>
         </is>
       </c>
-      <c r="H5" s="32" t="n"/>
-    </row>
-    <row r="6" ht="25" customHeight="1">
+    </row>
+    <row r="6">
       <c r="A6" s="8">
         <f>COUNTA(DADOS!A:A)-1</f>
         <v/>
       </c>
-      <c r="B6" s="32" t="n"/>
       <c r="C6" s="8">
         <f>COUNTIF(DADOS!S:S,"EM PRODUÇÃO")</f>
         <v/>
       </c>
-      <c r="D6" s="32" t="n"/>
       <c r="E6" s="8">
         <f>COUNTIF(DADOS!S:S,"ATRASADO")</f>
         <v/>
       </c>
-      <c r="F6" s="32" t="n"/>
       <c r="G6" s="8">
         <f>COUNTIF(DADOS!S:S,"CONCLUÍDO")</f>
         <v/>
       </c>
-      <c r="H6" s="32" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="33" t="n"/>
-      <c r="C7" s="33" t="n"/>
-      <c r="E7" s="33" t="n"/>
-      <c r="G7" s="33" t="n"/>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="34" t="inlineStr">
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>TOTAL CAIXAS</t>
         </is>
       </c>
-      <c r="B8" s="35" t="n"/>
-      <c r="C8" s="35" t="n"/>
-      <c r="D8" s="35" t="n"/>
-      <c r="E8" s="35" t="n"/>
-      <c r="F8" s="35" t="n"/>
-      <c r="G8" s="35" t="n"/>
-      <c r="H8" s="32" t="n"/>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>HORAS PLANEJADAS</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>HORAS ATRASO</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>OPs C/ ATRASO</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="36">
+      <c r="A9" s="8">
         <f>SUM(DADOS!F:F)</f>
         <v/>
       </c>
-      <c r="B9" s="37" t="n"/>
-      <c r="C9" s="36">
+      <c r="C9" s="8">
         <f>SUM(DADOS!P:P)</f>
         <v/>
       </c>
-      <c r="D9" s="37" t="n"/>
-      <c r="E9" s="36">
+      <c r="E9" s="8">
         <f>SUM(DADOS!T:T)</f>
         <v/>
       </c>
-      <c r="F9" s="37" t="n"/>
-      <c r="G9" s="36">
+      <c r="G9" s="8">
         <f>COUNTIF(DADOS!T:T,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H9" s="37" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="38" t="n"/>
-      <c r="B10" s="38" t="n"/>
-      <c r="C10" s="38" t="n"/>
-      <c r="D10" s="38" t="n"/>
-      <c r="E10" s="38" t="n"/>
-      <c r="F10" s="38" t="n"/>
-      <c r="G10" s="38" t="n"/>
-      <c r="H10" s="38" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="39" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>ALERTAS E NOTIFICAÇÕES</t>
         </is>
       </c>
-      <c r="B11" s="38" t="n"/>
-      <c r="C11" s="38" t="n"/>
-      <c r="D11" s="38" t="n"/>
-      <c r="E11" s="38" t="n"/>
-      <c r="F11" s="38" t="n"/>
-      <c r="G11" s="38" t="n"/>
-      <c r="H11" s="38" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
@@ -1023,23 +733,9 @@
           <t>• Nenhuma alerta no momento</t>
         </is>
       </c>
-      <c r="B12" s="35" t="n"/>
-      <c r="C12" s="35" t="n"/>
-      <c r="D12" s="35" t="n"/>
-      <c r="E12" s="35" t="n"/>
-      <c r="F12" s="35" t="n"/>
-      <c r="G12" s="35" t="n"/>
-      <c r="H12" s="32" t="n"/>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="40" t="inlineStr"/>
-      <c r="B13" s="35" t="n"/>
-      <c r="C13" s="35" t="n"/>
-      <c r="D13" s="35" t="n"/>
-      <c r="E13" s="35" t="n"/>
-      <c r="F13" s="35" t="n"/>
-      <c r="G13" s="35" t="n"/>
-      <c r="H13" s="32" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
@@ -1047,13 +743,6 @@
           <t>• O sistema está operacional</t>
         </is>
       </c>
-      <c r="B14" s="35" t="n"/>
-      <c r="C14" s="35" t="n"/>
-      <c r="D14" s="35" t="n"/>
-      <c r="E14" s="35" t="n"/>
-      <c r="F14" s="35" t="n"/>
-      <c r="G14" s="35" t="n"/>
-      <c r="H14" s="32" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
@@ -1061,13 +750,6 @@
           <t>• Clique nos botões abaixo para acessar as funcionalidades</t>
         </is>
       </c>
-      <c r="B15" s="35" t="n"/>
-      <c r="C15" s="35" t="n"/>
-      <c r="D15" s="35" t="n"/>
-      <c r="E15" s="35" t="n"/>
-      <c r="F15" s="35" t="n"/>
-      <c r="G15" s="35" t="n"/>
-      <c r="H15" s="32" t="n"/>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="11" t="inlineStr">
@@ -1082,17 +764,11 @@
           <t>📅 PLANEJAMENTO</t>
         </is>
       </c>
-      <c r="B20" s="41" t="n"/>
-      <c r="C20" s="41" t="n"/>
-      <c r="D20" s="42" t="n"/>
       <c r="E20" s="13" t="inlineStr">
         <is>
           <t>📋 OPERAÇÕES</t>
         </is>
       </c>
-      <c r="F20" s="41" t="n"/>
-      <c r="G20" s="41" t="n"/>
-      <c r="H20" s="42" t="n"/>
     </row>
     <row r="22" ht="6.666666666666667" customHeight="1">
       <c r="A22" s="13" t="inlineStr">
@@ -1100,20 +776,14 @@
           <t>⚙ MÁQUINAS</t>
         </is>
       </c>
-      <c r="B22" s="41" t="n"/>
-      <c r="C22" s="41" t="n"/>
-      <c r="D22" s="42" t="n"/>
       <c r="E22" s="13" t="inlineStr">
         <is>
           <t>🔎 PESQUISAR OP</t>
         </is>
       </c>
-      <c r="F22" s="41" t="n"/>
-      <c r="G22" s="41" t="n"/>
-      <c r="H22" s="42" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="30">
+  <mergeCells count="29">
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A15:H15"/>
     <mergeCell ref="A22:D22"/>
@@ -1139,7 +809,6 @@
     <mergeCell ref="E20:H20"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A8:H8"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="A13:H13"/>
     <mergeCell ref="A9:B9"/>
@@ -1169,29 +838,29 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Z14"/>
+  <dimension ref="A1:Z11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="14" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
     <col width="14" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="20" max="20"/>
     <col width="10" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="16" customWidth="1" min="23" max="23"/>
@@ -1199,22 +868,22 @@
     <col width="25" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="43" t="inlineStr">
+    <row r="1" ht="35" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>OPERAÇÕES</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="28" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>Gestão de ordens de produção</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="44" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>🔎 PESQUISAR OP</t>
         </is>
@@ -1246,55 +915,37 @@
       </c>
       <c r="H5" s="17" t="n"/>
     </row>
-    <row r="6">
-      <c r="A6" s="45" t="n"/>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="46" t="inlineStr">
-        <is>
-          <t>Numero da OP:</t>
-        </is>
-      </c>
-      <c r="B7" s="47" t="n"/>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="48" t="inlineStr">
-        <is>
-          <t>Produto:</t>
-        </is>
-      </c>
-      <c r="B8" s="49" t="n"/>
-      <c r="C8" s="42" t="n"/>
+    <row r="7">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>AÇÕES</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>+ NOVA OP</t>
+        </is>
+      </c>
       <c r="D8" s="18" t="inlineStr">
         <is>
           <t>🔄 ATUALIZAR</t>
         </is>
       </c>
-      <c r="E8" s="41" t="n"/>
-      <c r="F8" s="42" t="n"/>
       <c r="G8" s="18" t="inlineStr">
         <is>
           <t>← VOLTAR</t>
         </is>
       </c>
-      <c r="H8" s="41" t="n"/>
-      <c r="I8" s="42" t="n"/>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="50" t="inlineStr">
-        <is>
-          <t>Maquina:</t>
-        </is>
-      </c>
-      <c r="B9" s="47" t="n"/>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="51" t="inlineStr">
-        <is>
-          <t>Quantidade:</t>
-        </is>
-      </c>
-      <c r="B10" s="52" t="inlineStr">
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Produto</t>
         </is>
@@ -1415,13 +1066,13 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="53" t="inlineStr">
-        <is>
-          <t>Unidade:</t>
-        </is>
-      </c>
-      <c r="B11" s="54" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>OP001</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
         <is>
           <t>PURAN</t>
         </is>
@@ -1498,34 +1149,15 @@
       <c r="X11" s="19" t="inlineStr"/>
       <c r="Y11" s="12" t="inlineStr"/>
     </row>
-    <row r="12" ht="28" customHeight="1">
-      <c r="A12" s="55" t="inlineStr">
-        <is>
-          <t>SALVAR OP</t>
-        </is>
-      </c>
-      <c r="C12" s="56" t="inlineStr">
-        <is>
-          <t>CANCELAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="57" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="C12:D12"/>
+  <mergeCells count="7">
     <mergeCell ref="A1:Z1"/>
     <mergeCell ref="A7:H7"/>
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="G8:I8"/>
-    <mergeCell ref="A6:E6"/>
     <mergeCell ref="A2:Z2"/>
     <mergeCell ref="D8:F8"/>
-    <mergeCell ref="A14:T14"/>
-    <mergeCell ref="A12:B12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -1538,60 +1170,47 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Z13"/>
+  <dimension ref="A1:Z9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="43" t="inlineStr">
+    <row r="1" ht="35" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>MÁQUINAS</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="28" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>Gestão de recursos produtivos</t>
         </is>
       </c>
     </row>
     <row r="4" ht="25" customHeight="1">
-      <c r="A4" s="58" t="inlineStr">
+      <c r="A4" s="23" t="inlineStr">
         <is>
           <t>+ NOVA MÁQUINA</t>
         </is>
       </c>
-      <c r="B4" s="41" t="n"/>
-      <c r="C4" s="41" t="n"/>
-      <c r="D4" s="41" t="n"/>
-      <c r="E4" s="41" t="n"/>
-      <c r="F4" s="42" t="n"/>
-    </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="50" t="inlineStr">
-        <is>
-          <t>Codigo:</t>
-        </is>
-      </c>
-      <c r="B5" s="47" t="n"/>
-    </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="51" t="inlineStr">
-        <is>
-          <t>Nome:</t>
-        </is>
-      </c>
-      <c r="B6" s="52" t="inlineStr">
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Máquina</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Velocidade</t>
         </is>
@@ -1627,13 +1246,13 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="53" t="inlineStr">
-        <is>
-          <t>Velocidade (cx/h):</t>
-        </is>
-      </c>
-      <c r="B7" s="59" t="n">
+    <row r="7">
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>FETTE 2090</t>
+        </is>
+      </c>
+      <c r="B7" s="21" t="n">
         <v>500</v>
       </c>
       <c r="C7" s="21" t="inlineStr">
@@ -1661,13 +1280,13 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="53" t="inlineStr">
-        <is>
-          <t>OEE (%):</t>
-        </is>
-      </c>
-      <c r="B8" s="59" t="n">
+    <row r="8">
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>FETTE 2</t>
+        </is>
+      </c>
+      <c r="B8" s="21" t="n">
         <v>450</v>
       </c>
       <c r="C8" s="21" t="inlineStr">
@@ -1695,13 +1314,13 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="53" t="inlineStr">
-        <is>
-          <t>Setup (h):</t>
-        </is>
-      </c>
-      <c r="B9" s="59" t="n">
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>MEDISEAL</t>
+        </is>
+      </c>
+      <c r="B9" s="21" t="n">
         <v>600</v>
       </c>
       <c r="C9" s="21" t="inlineStr">
@@ -1729,27 +1348,9 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="28" customHeight="1">
-      <c r="A11" s="55" t="inlineStr">
-        <is>
-          <t>SALVAR MAQUINA</t>
-        </is>
-      </c>
-      <c r="C11" s="56" t="inlineStr">
-        <is>
-          <t>CANCELAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="57" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="3">
     <mergeCell ref="A1:Z1"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A13:H13"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="A2:Z2"/>
   </mergeCells>
@@ -1764,7 +1365,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CU9"/>
+  <dimension ref="A1:AW9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1818,70 +1419,19 @@
     <col width="9" customWidth="1" min="49" max="49"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="43" t="inlineStr">
+    <row r="1" ht="35" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>PLANEJAMENTO DA PRODUÇÃO</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="28" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>Timeline visual e cards das OPs</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="60" t="n"/>
-      <c r="B3" s="60" t="n"/>
-      <c r="C3" s="60" t="n"/>
-      <c r="D3" s="60" t="n"/>
-      <c r="E3" s="60" t="n"/>
-      <c r="F3" s="60" t="n"/>
-      <c r="G3" s="60" t="n"/>
-      <c r="H3" s="60" t="n"/>
-      <c r="I3" s="60" t="n"/>
-      <c r="J3" s="60" t="n"/>
-      <c r="K3" s="60" t="n"/>
-      <c r="L3" s="60" t="n"/>
-      <c r="M3" s="60" t="n"/>
-      <c r="N3" s="60" t="n"/>
-      <c r="O3" s="60" t="n"/>
-      <c r="P3" s="60" t="n"/>
-      <c r="Q3" s="60" t="n"/>
-      <c r="R3" s="60" t="n"/>
-      <c r="S3" s="60" t="n"/>
-      <c r="T3" s="60" t="n"/>
-      <c r="U3" s="60" t="n"/>
-      <c r="V3" s="60" t="n"/>
-      <c r="W3" s="60" t="n"/>
-      <c r="X3" s="60" t="n"/>
-      <c r="Y3" s="60" t="n"/>
-      <c r="Z3" s="60" t="n"/>
-      <c r="AA3" s="60" t="n"/>
-      <c r="AB3" s="60" t="n"/>
-      <c r="AC3" s="60" t="n"/>
-      <c r="AD3" s="60" t="n"/>
-      <c r="AE3" s="60" t="n"/>
-      <c r="AF3" s="60" t="n"/>
-      <c r="AG3" s="60" t="n"/>
-      <c r="AH3" s="60" t="n"/>
-      <c r="AI3" s="60" t="n"/>
-      <c r="AJ3" s="60" t="n"/>
-      <c r="AK3" s="60" t="n"/>
-      <c r="AL3" s="60" t="n"/>
-      <c r="AM3" s="60" t="n"/>
-      <c r="AN3" s="60" t="n"/>
-      <c r="AO3" s="60" t="n"/>
-      <c r="AP3" s="60" t="n"/>
-      <c r="AQ3" s="60" t="n"/>
-      <c r="AR3" s="60" t="n"/>
-      <c r="AS3" s="60" t="n"/>
-      <c r="AT3" s="60" t="n"/>
-      <c r="AU3" s="60" t="n"/>
-      <c r="AV3" s="60" t="n"/>
-      <c r="AW3" s="60" t="n"/>
     </row>
     <row r="4" ht="25" customHeight="1">
       <c r="A4" s="18" t="inlineStr">
@@ -1889,21 +1439,6 @@
           <t>🔄 RECALCULAR  ⚠ ATRASOS  🔧 EVENTOS  🍽 REFEIÇÕES  🏠 DASHBOARD</t>
         </is>
       </c>
-      <c r="B4" s="41" t="n"/>
-      <c r="C4" s="41" t="n"/>
-      <c r="D4" s="41" t="n"/>
-      <c r="E4" s="41" t="n"/>
-      <c r="F4" s="41" t="n"/>
-      <c r="G4" s="41" t="n"/>
-      <c r="H4" s="41" t="n"/>
-      <c r="I4" s="41" t="n"/>
-      <c r="J4" s="41" t="n"/>
-      <c r="K4" s="41" t="n"/>
-      <c r="L4" s="41" t="n"/>
-      <c r="M4" s="41" t="n"/>
-      <c r="N4" s="41" t="n"/>
-      <c r="O4" s="41" t="n"/>
-      <c r="P4" s="42" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="25" t="inlineStr">
@@ -2174,10 +1709,8 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A2:CU2"/>
+  <mergeCells count="3">
     <mergeCell ref="A1:Z1"/>
-    <mergeCell ref="A1:CU1"/>
     <mergeCell ref="A4:P4"/>
     <mergeCell ref="A2:Z2"/>
   </mergeCells>

</xml_diff>